<commit_message>
project done ( integration of the final model )
</commit_message>
<xml_diff>
--- a/Model/fichiers pour tester le model/Version 1/clients.xlsx
+++ b/Model/fichiers pour tester le model/Version 1/clients.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CHAKIR\Model\fichiers pour tester le model\Version 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{858B519D-387F-4AE9-AA00-305BE698AAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8C030C-9ECA-4ACA-9DD0-EF40AE8FA8F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="121">
   <si>
     <t>Subs_Id</t>
   </si>
@@ -264,24 +264,6 @@
     <t>REV_M6</t>
   </si>
   <si>
-    <t>top1_usage</t>
-  </si>
-  <si>
-    <t>top2_usage</t>
-  </si>
-  <si>
-    <t>top3_usage</t>
-  </si>
-  <si>
-    <t>top1_revenue</t>
-  </si>
-  <si>
-    <t>top2_revenue</t>
-  </si>
-  <si>
-    <t>top3_revenue</t>
-  </si>
-  <si>
     <t>Tenure</t>
   </si>
   <si>
@@ -291,9 +273,6 @@
     <t>Offre Data Plus</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>1002</t>
   </si>
   <si>
@@ -318,9 +297,6 @@
     <t>Offre Basic</t>
   </si>
   <si>
-    <t>Inactive</t>
-  </si>
-  <si>
     <t>1005</t>
   </si>
   <si>
@@ -403,6 +379,15 @@
   </si>
   <si>
     <t>LV</t>
+  </si>
+  <si>
+    <t>Tenure_Segment</t>
+  </si>
+  <si>
+    <t>More than 5 years</t>
+  </si>
+  <si>
+    <t>Between 3 and 5 years</t>
   </si>
 </sst>
 </file>
@@ -787,7 +772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CI11"/>
+  <dimension ref="A1:CD11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -827,12 +812,13 @@
     <col min="72" max="72" width="23" customWidth="1"/>
     <col min="73" max="73" width="22" customWidth="1"/>
     <col min="74" max="79" width="12" customWidth="1"/>
-    <col min="80" max="82" width="13" customWidth="1"/>
+    <col min="80" max="81" width="13" customWidth="1"/>
+    <col min="82" max="82" width="20.33203125" customWidth="1"/>
     <col min="83" max="85" width="15" customWidth="1"/>
     <col min="86" max="86" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -840,7 +826,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1076,49 +1062,34 @@
       <c r="CC1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="CD1" s="1" t="s">
+      <c r="CD1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:82" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="CE1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="CF1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="CG1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="CH1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="CI1" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:87" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2">
         <v>2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2">
         <v>350</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>88</v>
+      <c r="G2" s="2">
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="I2" s="2">
         <v>0</v>
@@ -1337,51 +1308,36 @@
         <v>561.71</v>
       </c>
       <c r="CC2" s="2">
-        <v>180</v>
-      </c>
-      <c r="CD2" s="2">
-        <v>157.5</v>
-      </c>
-      <c r="CE2" s="2">
-        <v>112.5</v>
-      </c>
-      <c r="CF2" s="2">
-        <v>202.5</v>
-      </c>
-      <c r="CG2" s="2">
-        <v>135</v>
-      </c>
-      <c r="CH2" s="2">
-        <v>112.5</v>
-      </c>
-      <c r="CI2" s="2">
         <v>36</v>
       </c>
+      <c r="CD2" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="3" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D3" s="3">
         <v>8</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F3" s="3">
         <v>150</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>88</v>
+      <c r="G3" s="3">
+        <v>1</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="I3" s="3">
         <v>0.1</v>
@@ -1600,51 +1556,36 @@
         <v>229.78</v>
       </c>
       <c r="CC3" s="3">
-        <v>112</v>
-      </c>
-      <c r="CD3" s="3">
-        <v>98</v>
-      </c>
-      <c r="CE3" s="3">
-        <v>70</v>
-      </c>
-      <c r="CF3" s="3">
-        <v>126</v>
-      </c>
-      <c r="CG3" s="3">
-        <v>84</v>
-      </c>
-      <c r="CH3" s="3">
-        <v>70</v>
-      </c>
-      <c r="CI3" s="3">
         <v>24</v>
       </c>
+      <c r="CD3" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="4" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F4" s="2">
         <v>350</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>88</v>
+      <c r="G4" s="2">
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="I4" s="2">
         <v>0</v>
@@ -1863,51 +1804,36 @@
         <v>457.15</v>
       </c>
       <c r="CC4" s="2">
-        <v>240</v>
-      </c>
-      <c r="CD4" s="2">
-        <v>210</v>
-      </c>
-      <c r="CE4" s="2">
-        <v>150</v>
-      </c>
-      <c r="CF4" s="2">
-        <v>270</v>
-      </c>
-      <c r="CG4" s="2">
-        <v>180</v>
-      </c>
-      <c r="CH4" s="2">
-        <v>150</v>
-      </c>
-      <c r="CI4" s="2">
         <v>48</v>
       </c>
+      <c r="CD4" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="5" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F5" s="3">
         <v>200</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>97</v>
+      <c r="G5" s="3">
+        <v>0</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="I5" s="3">
         <v>0.8</v>
@@ -2126,51 +2052,36 @@
         <v>76.540000000000006</v>
       </c>
       <c r="CC5" s="3">
-        <v>32</v>
-      </c>
-      <c r="CD5" s="3">
-        <v>28</v>
-      </c>
-      <c r="CE5" s="3">
-        <v>20</v>
-      </c>
-      <c r="CF5" s="3">
-        <v>36</v>
-      </c>
-      <c r="CG5" s="3">
-        <v>24</v>
-      </c>
-      <c r="CH5" s="3">
-        <v>20</v>
-      </c>
-      <c r="CI5" s="3">
         <v>12</v>
       </c>
+      <c r="CD5" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="6" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D6" s="2">
         <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F6" s="2">
         <v>200</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>88</v>
+      <c r="G6" s="2">
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="I6" s="2">
         <v>0.2</v>
@@ -2389,51 +2300,36 @@
         <v>372.13</v>
       </c>
       <c r="CC6" s="2">
-        <v>128</v>
-      </c>
-      <c r="CD6" s="2">
-        <v>112</v>
-      </c>
-      <c r="CE6" s="2">
-        <v>80</v>
-      </c>
-      <c r="CF6" s="2">
-        <v>144</v>
-      </c>
-      <c r="CG6" s="2">
-        <v>96</v>
-      </c>
-      <c r="CH6" s="2">
-        <v>80</v>
-      </c>
-      <c r="CI6" s="2">
         <v>30</v>
       </c>
+      <c r="CD6" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="7" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D7" s="3">
         <v>2</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F7" s="3">
         <v>350</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>88</v>
+      <c r="G7" s="3">
+        <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="I7" s="3">
         <v>0</v>
@@ -2652,51 +2548,36 @@
         <v>447.21</v>
       </c>
       <c r="CC7" s="3">
-        <v>200</v>
-      </c>
-      <c r="CD7" s="3">
-        <v>175</v>
-      </c>
-      <c r="CE7" s="3">
-        <v>125</v>
-      </c>
-      <c r="CF7" s="3">
-        <v>225</v>
-      </c>
-      <c r="CG7" s="3">
-        <v>150</v>
-      </c>
-      <c r="CH7" s="3">
-        <v>125</v>
-      </c>
-      <c r="CI7" s="3">
         <v>60</v>
       </c>
+      <c r="CD7" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="8" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D8" s="2">
         <v>1</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F8" s="2">
         <v>200</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>97</v>
+      <c r="G8" s="2">
+        <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="I8" s="2">
         <v>0.9</v>
@@ -2915,51 +2796,36 @@
         <v>61.64</v>
       </c>
       <c r="CC8" s="2">
-        <v>20</v>
-      </c>
-      <c r="CD8" s="2">
-        <v>17.5</v>
-      </c>
-      <c r="CE8" s="2">
-        <v>12.5</v>
-      </c>
-      <c r="CF8" s="2">
-        <v>22.5</v>
-      </c>
-      <c r="CG8" s="2">
-        <v>15</v>
-      </c>
-      <c r="CH8" s="2">
-        <v>12.5</v>
-      </c>
-      <c r="CI8" s="2">
         <v>6</v>
       </c>
+      <c r="CD8" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="9" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D9" s="3">
         <v>8</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F9" s="3">
         <v>150</v>
       </c>
-      <c r="G9" s="3" t="s">
-        <v>88</v>
+      <c r="G9" s="3">
+        <v>1</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="I9" s="3">
         <v>0.1</v>
@@ -3178,51 +3044,36 @@
         <v>247.22</v>
       </c>
       <c r="CC9" s="3">
-        <v>140</v>
-      </c>
-      <c r="CD9" s="3">
-        <v>122.5</v>
-      </c>
-      <c r="CE9" s="3">
-        <v>87.5</v>
-      </c>
-      <c r="CF9" s="3">
-        <v>157.5</v>
-      </c>
-      <c r="CG9" s="3">
-        <v>105</v>
-      </c>
-      <c r="CH9" s="3">
-        <v>87.5</v>
-      </c>
-      <c r="CI9" s="3">
         <v>18</v>
       </c>
+      <c r="CD9" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="10" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D10" s="2">
         <v>8</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F10" s="2">
         <v>150</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>88</v>
+      <c r="G10" s="2">
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="I10" s="2">
         <v>0</v>
@@ -3441,51 +3292,36 @@
         <v>703.25</v>
       </c>
       <c r="CC10" s="2">
-        <v>280</v>
-      </c>
-      <c r="CD10" s="2">
-        <v>245</v>
-      </c>
-      <c r="CE10" s="2">
-        <v>175</v>
-      </c>
-      <c r="CF10" s="2">
-        <v>315</v>
-      </c>
-      <c r="CG10" s="2">
-        <v>210</v>
-      </c>
-      <c r="CH10" s="2">
-        <v>175</v>
-      </c>
-      <c r="CI10" s="2">
         <v>54</v>
       </c>
+      <c r="CD10" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="11" spans="1:87" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:82" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D11" s="3">
         <v>1</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F11" s="3">
         <v>200</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>88</v>
+      <c r="G11" s="3">
+        <v>1</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="I11" s="3">
         <v>0.3</v>
@@ -3704,25 +3540,10 @@
         <v>236.33</v>
       </c>
       <c r="CC11" s="3">
-        <v>80</v>
-      </c>
-      <c r="CD11" s="3">
-        <v>70</v>
-      </c>
-      <c r="CE11" s="3">
-        <v>50</v>
-      </c>
-      <c r="CF11" s="3">
-        <v>90</v>
-      </c>
-      <c r="CG11" s="3">
-        <v>60</v>
-      </c>
-      <c r="CH11" s="3">
-        <v>50</v>
-      </c>
-      <c r="CI11" s="3">
         <v>15</v>
+      </c>
+      <c r="CD11" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>